<commit_message>
Value-binding method and referenceEvaluation names are written with spaces (horizontal offset, sequence between, volume top, ...): dropdown lists in the dictionary workbooks and the template, and the designProperty and properties dictionaries regenerated.
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/conditionOnReceipt.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/conditionOnReceipt.xlsx
@@ -2276,13 +2276,13 @@
   </sheetData>
   <dataValidations count="3">
     <dataValidation sqref="D2:D31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"direct,horizontal_offset,difference,reverse_difference,angular_difference,containment,sequence_between,value_at,rate,rate_per_log_cycle,within_envelope,frequency"</formula1>
+      <formula1>"direct,horizontal offset,difference,reverse difference,angular difference,containment,sequence between,value at,rate,rate per log cycle,within envelope,frequency"</formula1>
     </dataValidation>
     <dataValidation sqref="G2:G31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"design,evidence"</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"value,vertical_intersection,volume_top,volume_base"</formula1>
+      <formula1>"value,vertical intersection,volume top,volume base"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>